<commit_message>
sigh fix the diode p/n
</commit_message>
<xml_diff>
--- a/TURFv6/revC/TURFv6_revC_BOM_041525.xlsx
+++ b/TURFv6/revC/TURFv6_revC_BOM_041525.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\pueo-daq-design\TURFv6\revC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EECFFCB-E100-435C-AE6A-156FCECF6241}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFC5FD8E-8B9F-4092-BD39-6F825523019F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D3B74482-F8A5-4E82-A69B-8579953A21D8}"/>
   </bookViews>
@@ -266,15 +266,9 @@
     <t>DT1446</t>
   </si>
   <si>
-    <t>DT1446-04TS-7</t>
-  </si>
-  <si>
     <t>Diodes, Inc.</t>
   </si>
   <si>
-    <t>ESD Suppressor Diode Array Uni-Dir 5V Automotive 6-Pin TSOT-26 T/R</t>
-  </si>
-  <si>
     <t>J17</t>
   </si>
   <si>
@@ -921,6 +915,12 @@
   </si>
   <si>
     <t>MOSFET N-CH 60V 115MA SOT23-3</t>
+  </si>
+  <si>
+    <t>DT1446-04S-7</t>
+  </si>
+  <si>
+    <t>8.5V Clamp 4.7A (8/20µs) Ipp Tvs Diode Surface Mount SOT-363</t>
   </si>
 </sst>
 </file>
@@ -1404,7 +1404,7 @@
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D5" t="s">
         <v>19</v>
@@ -1413,10 +1413,10 @@
         <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="G5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
@@ -1502,7 +1502,7 @@
         <v>33</v>
       </c>
       <c r="E9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="F9" t="s">
         <v>17</v>
@@ -1631,19 +1631,19 @@
         <v>18</v>
       </c>
       <c r="C15" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D15" t="s">
         <v>49</v>
       </c>
       <c r="E15" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G15" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1654,16 +1654,16 @@
         <v>44</v>
       </c>
       <c r="C16" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D16" t="s">
         <v>49</v>
       </c>
       <c r="E16" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="F16" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G16" t="s">
         <v>50</v>
@@ -1677,19 +1677,19 @@
         <v>3</v>
       </c>
       <c r="C17" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D17" t="s">
         <v>52</v>
       </c>
       <c r="E17" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="F17" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G17" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
@@ -1706,13 +1706,13 @@
         <v>54</v>
       </c>
       <c r="E18" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F18" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="G18" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
@@ -1723,16 +1723,16 @@
         <v>6</v>
       </c>
       <c r="C19" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D19" t="s">
         <v>55</v>
       </c>
       <c r="E19" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="F19" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G19" t="s">
         <v>56</v>
@@ -1746,19 +1746,19 @@
         <v>2</v>
       </c>
       <c r="C20" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D20" t="s">
         <v>57</v>
       </c>
       <c r="E20" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="F20" t="s">
         <v>51</v>
       </c>
       <c r="G20" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
@@ -1769,19 +1769,19 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D21" t="s">
         <v>58</v>
       </c>
       <c r="E21" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="F21" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="G21" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
@@ -1798,13 +1798,13 @@
         <v>60</v>
       </c>
       <c r="E22" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="F22" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="G22" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
@@ -1913,13 +1913,13 @@
         <v>75</v>
       </c>
       <c r="E27" t="s">
+        <v>293</v>
+      </c>
+      <c r="F27" t="s">
         <v>76</v>
       </c>
-      <c r="F27" t="s">
-        <v>77</v>
-      </c>
       <c r="G27" t="s">
-        <v>78</v>
+        <v>294</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
@@ -1930,19 +1930,19 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
+        <v>77</v>
+      </c>
+      <c r="D28" t="s">
+        <v>78</v>
+      </c>
+      <c r="E28" t="s">
+        <v>78</v>
+      </c>
+      <c r="F28" t="s">
         <v>79</v>
       </c>
-      <c r="D28" t="s">
+      <c r="G28" t="s">
         <v>80</v>
-      </c>
-      <c r="E28" t="s">
-        <v>80</v>
-      </c>
-      <c r="F28" t="s">
-        <v>81</v>
-      </c>
-      <c r="G28" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
@@ -1953,19 +1953,19 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F29" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G29" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
@@ -1976,19 +1976,19 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
+        <v>83</v>
+      </c>
+      <c r="D30" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" t="s">
         <v>85</v>
       </c>
-      <c r="D30" t="s">
+      <c r="F30" t="s">
         <v>86</v>
       </c>
-      <c r="E30" t="s">
+      <c r="G30" t="s">
         <v>87</v>
-      </c>
-      <c r="F30" t="s">
-        <v>88</v>
-      </c>
-      <c r="G30" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
@@ -1999,10 +1999,10 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E31" t="s">
         <v>9</v>
@@ -2022,10 +2022,10 @@
         <v>2</v>
       </c>
       <c r="C32" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D32" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E32" t="s">
         <v>9</v>
@@ -2045,19 +2045,19 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
+        <v>92</v>
+      </c>
+      <c r="D33" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" t="s">
         <v>94</v>
       </c>
-      <c r="D33" t="s">
+      <c r="F33" t="s">
         <v>95</v>
       </c>
-      <c r="E33" t="s">
+      <c r="G33" t="s">
         <v>96</v>
-      </c>
-      <c r="F33" t="s">
-        <v>97</v>
-      </c>
-      <c r="G33" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
@@ -2068,19 +2068,19 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D34" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E34" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F34" t="s">
         <v>41</v>
       </c>
       <c r="G34" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
@@ -2091,19 +2091,19 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
+        <v>100</v>
+      </c>
+      <c r="D35" t="s">
+        <v>101</v>
+      </c>
+      <c r="E35" t="s">
+        <v>289</v>
+      </c>
+      <c r="F35" t="s">
         <v>102</v>
       </c>
-      <c r="D35" t="s">
+      <c r="G35" t="s">
         <v>103</v>
-      </c>
-      <c r="E35" t="s">
-        <v>291</v>
-      </c>
-      <c r="F35" t="s">
-        <v>104</v>
-      </c>
-      <c r="G35" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
@@ -2114,19 +2114,19 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
+        <v>104</v>
+      </c>
+      <c r="D36" t="s">
+        <v>105</v>
+      </c>
+      <c r="E36" t="s">
         <v>106</v>
-      </c>
-      <c r="D36" t="s">
-        <v>107</v>
-      </c>
-      <c r="E36" t="s">
-        <v>108</v>
       </c>
       <c r="F36" t="s">
         <v>17</v>
       </c>
       <c r="G36" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
@@ -2137,19 +2137,19 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D37" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E37" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F37" t="s">
         <v>17</v>
       </c>
       <c r="G37" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
@@ -2160,10 +2160,10 @@
         <v>2</v>
       </c>
       <c r="C38" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D38" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E38" t="s">
         <v>9</v>
@@ -2183,10 +2183,10 @@
         <v>2</v>
       </c>
       <c r="C39" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D39" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E39" t="s">
         <v>9</v>
@@ -2206,19 +2206,19 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
+        <v>115</v>
+      </c>
+      <c r="D40" t="s">
+        <v>116</v>
+      </c>
+      <c r="E40" t="s">
+        <v>116</v>
+      </c>
+      <c r="F40" t="s">
         <v>117</v>
       </c>
-      <c r="D40" t="s">
+      <c r="G40" t="s">
         <v>118</v>
-      </c>
-      <c r="E40" t="s">
-        <v>118</v>
-      </c>
-      <c r="F40" t="s">
-        <v>119</v>
-      </c>
-      <c r="G40" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
@@ -2229,10 +2229,10 @@
         <v>28</v>
       </c>
       <c r="C41" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D41" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="E41" t="s">
         <v>9</v>
@@ -2252,19 +2252,19 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
+        <v>121</v>
+      </c>
+      <c r="D42" t="s">
+        <v>122</v>
+      </c>
+      <c r="E42" t="s">
+        <v>122</v>
+      </c>
+      <c r="F42" t="s">
         <v>123</v>
       </c>
-      <c r="D42" t="s">
+      <c r="G42" t="s">
         <v>124</v>
-      </c>
-      <c r="E42" t="s">
-        <v>124</v>
-      </c>
-      <c r="F42" t="s">
-        <v>125</v>
-      </c>
-      <c r="G42" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -2275,19 +2275,19 @@
         <v>2</v>
       </c>
       <c r="C43" t="s">
+        <v>125</v>
+      </c>
+      <c r="D43" t="s">
+        <v>126</v>
+      </c>
+      <c r="E43" t="s">
         <v>127</v>
-      </c>
-      <c r="D43" t="s">
-        <v>128</v>
-      </c>
-      <c r="E43" t="s">
-        <v>129</v>
       </c>
       <c r="F43" t="s">
         <v>51</v>
       </c>
       <c r="G43" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -2298,19 +2298,19 @@
         <v>1</v>
       </c>
       <c r="C44" t="s">
+        <v>129</v>
+      </c>
+      <c r="D44" t="s">
+        <v>130</v>
+      </c>
+      <c r="E44" t="s">
         <v>131</v>
       </c>
-      <c r="D44" t="s">
+      <c r="F44" t="s">
         <v>132</v>
       </c>
-      <c r="E44" t="s">
+      <c r="G44" t="s">
         <v>133</v>
-      </c>
-      <c r="F44" t="s">
-        <v>134</v>
-      </c>
-      <c r="G44" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
@@ -2321,19 +2321,19 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
+        <v>134</v>
+      </c>
+      <c r="D45" t="s">
+        <v>135</v>
+      </c>
+      <c r="E45" t="s">
         <v>136</v>
       </c>
-      <c r="D45" t="s">
+      <c r="F45" t="s">
+        <v>132</v>
+      </c>
+      <c r="G45" t="s">
         <v>137</v>
-      </c>
-      <c r="E45" t="s">
-        <v>138</v>
-      </c>
-      <c r="F45" t="s">
-        <v>134</v>
-      </c>
-      <c r="G45" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -2344,19 +2344,19 @@
         <v>2</v>
       </c>
       <c r="C46" t="s">
+        <v>138</v>
+      </c>
+      <c r="D46" t="s">
+        <v>139</v>
+      </c>
+      <c r="E46" t="s">
+        <v>288</v>
+      </c>
+      <c r="F46" t="s">
+        <v>79</v>
+      </c>
+      <c r="G46" t="s">
         <v>140</v>
-      </c>
-      <c r="D46" t="s">
-        <v>141</v>
-      </c>
-      <c r="E46" t="s">
-        <v>290</v>
-      </c>
-      <c r="F46" t="s">
-        <v>81</v>
-      </c>
-      <c r="G46" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -2367,19 +2367,19 @@
         <v>5</v>
       </c>
       <c r="C47" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E47" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="F47" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G47" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
@@ -2390,19 +2390,19 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D48" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E48" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="F48" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G48" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
@@ -2413,19 +2413,19 @@
         <v>4</v>
       </c>
       <c r="C49" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D49" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E49" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F49" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G49" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -2436,19 +2436,19 @@
         <v>34</v>
       </c>
       <c r="C50" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D50" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E50" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F50" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G50" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
@@ -2459,19 +2459,19 @@
         <v>2</v>
       </c>
       <c r="C51" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D51" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E51" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="F51" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G51" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
@@ -2482,19 +2482,19 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D52" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E52" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="F52" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G52" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
@@ -2505,19 +2505,19 @@
         <v>2</v>
       </c>
       <c r="C53" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D53" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E53" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="F53" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="G53" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
@@ -2528,19 +2528,19 @@
         <v>2</v>
       </c>
       <c r="C54" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D54" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E54" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="F54" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G54" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
@@ -2551,19 +2551,19 @@
         <v>9</v>
       </c>
       <c r="C55" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D55" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E55" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="F55" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="G55" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
@@ -2574,19 +2574,19 @@
         <v>2</v>
       </c>
       <c r="C56" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D56" t="s">
+        <v>248</v>
+      </c>
+      <c r="E56" t="s">
+        <v>278</v>
+      </c>
+      <c r="F56" t="s">
+        <v>269</v>
+      </c>
+      <c r="G56" t="s">
         <v>250</v>
-      </c>
-      <c r="E56" t="s">
-        <v>280</v>
-      </c>
-      <c r="F56" t="s">
-        <v>271</v>
-      </c>
-      <c r="G56" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
@@ -2597,19 +2597,19 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="D57" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E57" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="F57" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G57" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
@@ -2620,19 +2620,19 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D58" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E58" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="F58" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G58" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
@@ -2643,19 +2643,19 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D59" t="s">
+        <v>249</v>
+      </c>
+      <c r="E59" t="s">
+        <v>282</v>
+      </c>
+      <c r="F59" t="s">
+        <v>269</v>
+      </c>
+      <c r="G59" t="s">
         <v>251</v>
-      </c>
-      <c r="E59" t="s">
-        <v>284</v>
-      </c>
-      <c r="F59" t="s">
-        <v>271</v>
-      </c>
-      <c r="G59" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
@@ -2666,19 +2666,19 @@
         <v>3</v>
       </c>
       <c r="C60" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="D60" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E60" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="F60" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G60" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
@@ -2689,19 +2689,19 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D61" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E61" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="F61" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G61" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
@@ -2712,10 +2712,10 @@
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D62" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E62" t="s">
         <v>9</v>
@@ -2735,19 +2735,19 @@
         <v>1</v>
       </c>
       <c r="C63" t="s">
+        <v>164</v>
+      </c>
+      <c r="D63" t="s">
+        <v>165</v>
+      </c>
+      <c r="E63" t="s">
         <v>166</v>
       </c>
-      <c r="D63" t="s">
+      <c r="F63" t="s">
         <v>167</v>
       </c>
-      <c r="E63" t="s">
+      <c r="G63" t="s">
         <v>168</v>
-      </c>
-      <c r="F63" t="s">
-        <v>169</v>
-      </c>
-      <c r="G63" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
@@ -2758,10 +2758,10 @@
         <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D64" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E64" t="s">
         <v>9</v>
@@ -2781,19 +2781,19 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
+        <v>170</v>
+      </c>
+      <c r="D65" t="s">
+        <v>171</v>
+      </c>
+      <c r="E65" t="s">
+        <v>246</v>
+      </c>
+      <c r="F65" t="s">
+        <v>247</v>
+      </c>
+      <c r="G65" t="s">
         <v>172</v>
-      </c>
-      <c r="D65" t="s">
-        <v>173</v>
-      </c>
-      <c r="E65" t="s">
-        <v>248</v>
-      </c>
-      <c r="F65" t="s">
-        <v>249</v>
-      </c>
-      <c r="G65" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
@@ -2804,19 +2804,19 @@
         <v>4</v>
       </c>
       <c r="C66" t="s">
+        <v>173</v>
+      </c>
+      <c r="D66" t="s">
+        <v>171</v>
+      </c>
+      <c r="E66" t="s">
+        <v>174</v>
+      </c>
+      <c r="F66" t="s">
         <v>175</v>
       </c>
-      <c r="D66" t="s">
-        <v>173</v>
-      </c>
-      <c r="E66" t="s">
+      <c r="G66" t="s">
         <v>176</v>
-      </c>
-      <c r="F66" t="s">
-        <v>177</v>
-      </c>
-      <c r="G66" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
@@ -2827,19 +2827,19 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
+        <v>177</v>
+      </c>
+      <c r="D67" t="s">
+        <v>178</v>
+      </c>
+      <c r="E67" t="s">
+        <v>178</v>
+      </c>
+      <c r="F67" t="s">
+        <v>102</v>
+      </c>
+      <c r="G67" t="s">
         <v>179</v>
-      </c>
-      <c r="D67" t="s">
-        <v>180</v>
-      </c>
-      <c r="E67" t="s">
-        <v>180</v>
-      </c>
-      <c r="F67" t="s">
-        <v>104</v>
-      </c>
-      <c r="G67" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
@@ -2850,19 +2850,19 @@
         <v>2</v>
       </c>
       <c r="C68" t="s">
+        <v>180</v>
+      </c>
+      <c r="D68" t="s">
+        <v>181</v>
+      </c>
+      <c r="E68" t="s">
+        <v>181</v>
+      </c>
+      <c r="F68" t="s">
+        <v>102</v>
+      </c>
+      <c r="G68" t="s">
         <v>182</v>
-      </c>
-      <c r="D68" t="s">
-        <v>183</v>
-      </c>
-      <c r="E68" t="s">
-        <v>183</v>
-      </c>
-      <c r="F68" t="s">
-        <v>104</v>
-      </c>
-      <c r="G68" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
@@ -2873,19 +2873,19 @@
         <v>3</v>
       </c>
       <c r="C69" t="s">
+        <v>183</v>
+      </c>
+      <c r="D69" t="s">
+        <v>184</v>
+      </c>
+      <c r="E69" t="s">
+        <v>184</v>
+      </c>
+      <c r="F69" t="s">
         <v>185</v>
       </c>
-      <c r="D69" t="s">
+      <c r="G69" t="s">
         <v>186</v>
-      </c>
-      <c r="E69" t="s">
-        <v>186</v>
-      </c>
-      <c r="F69" t="s">
-        <v>187</v>
-      </c>
-      <c r="G69" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
@@ -2896,19 +2896,19 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
+        <v>187</v>
+      </c>
+      <c r="D70" t="s">
+        <v>188</v>
+      </c>
+      <c r="E70" t="s">
         <v>189</v>
       </c>
-      <c r="D70" t="s">
+      <c r="F70" t="s">
+        <v>102</v>
+      </c>
+      <c r="G70" t="s">
         <v>190</v>
-      </c>
-      <c r="E70" t="s">
-        <v>191</v>
-      </c>
-      <c r="F70" t="s">
-        <v>104</v>
-      </c>
-      <c r="G70" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.3">
@@ -2919,19 +2919,19 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D71" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E71" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="F71" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G71" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
@@ -2942,10 +2942,10 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D72" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="E72" t="s">
         <v>9</v>
@@ -2965,19 +2965,19 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
+        <v>193</v>
+      </c>
+      <c r="D73" t="s">
+        <v>194</v>
+      </c>
+      <c r="E73" t="s">
+        <v>194</v>
+      </c>
+      <c r="F73" t="s">
+        <v>102</v>
+      </c>
+      <c r="G73" t="s">
         <v>195</v>
-      </c>
-      <c r="D73" t="s">
-        <v>196</v>
-      </c>
-      <c r="E73" t="s">
-        <v>196</v>
-      </c>
-      <c r="F73" t="s">
-        <v>104</v>
-      </c>
-      <c r="G73" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
@@ -2988,19 +2988,19 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D74" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="E74" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F74" t="s">
         <v>17</v>
       </c>
       <c r="G74" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
@@ -3011,19 +3011,19 @@
         <v>1</v>
       </c>
       <c r="C75" t="s">
+        <v>199</v>
+      </c>
+      <c r="D75" t="s">
+        <v>200</v>
+      </c>
+      <c r="E75" t="s">
+        <v>200</v>
+      </c>
+      <c r="F75" t="s">
         <v>201</v>
       </c>
-      <c r="D75" t="s">
+      <c r="G75" t="s">
         <v>202</v>
-      </c>
-      <c r="E75" t="s">
-        <v>202</v>
-      </c>
-      <c r="F75" t="s">
-        <v>203</v>
-      </c>
-      <c r="G75" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
@@ -3034,19 +3034,19 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
+        <v>203</v>
+      </c>
+      <c r="D76" t="s">
+        <v>204</v>
+      </c>
+      <c r="E76" t="s">
+        <v>204</v>
+      </c>
+      <c r="F76" t="s">
+        <v>201</v>
+      </c>
+      <c r="G76" t="s">
         <v>205</v>
-      </c>
-      <c r="D76" t="s">
-        <v>206</v>
-      </c>
-      <c r="E76" t="s">
-        <v>206</v>
-      </c>
-      <c r="F76" t="s">
-        <v>203</v>
-      </c>
-      <c r="G76" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
@@ -3057,19 +3057,19 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
+        <v>206</v>
+      </c>
+      <c r="D77" t="s">
+        <v>207</v>
+      </c>
+      <c r="E77" t="s">
         <v>208</v>
       </c>
-      <c r="D77" t="s">
+      <c r="F77" t="s">
         <v>209</v>
       </c>
-      <c r="E77" t="s">
+      <c r="G77" t="s">
         <v>210</v>
-      </c>
-      <c r="F77" t="s">
-        <v>211</v>
-      </c>
-      <c r="G77" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
@@ -3080,19 +3080,19 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
+        <v>211</v>
+      </c>
+      <c r="D78" t="s">
+        <v>212</v>
+      </c>
+      <c r="E78" t="s">
         <v>213</v>
       </c>
-      <c r="D78" t="s">
+      <c r="F78" t="s">
+        <v>209</v>
+      </c>
+      <c r="G78" t="s">
         <v>214</v>
-      </c>
-      <c r="E78" t="s">
-        <v>215</v>
-      </c>
-      <c r="F78" t="s">
-        <v>211</v>
-      </c>
-      <c r="G78" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
@@ -3103,7 +3103,7 @@
         <v>4</v>
       </c>
       <c r="C79" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D79" t="s">
         <v>19</v>
@@ -3115,7 +3115,7 @@
         <v>21</v>
       </c>
       <c r="G79" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
   </sheetData>

</xml_diff>